<commit_message>
feat: introduce additional tables
</commit_message>
<xml_diff>
--- a/output/five-decade-tables/ppbr_by_group - manual edit.xlsx
+++ b/output/five-decade-tables/ppbr_by_group - manual edit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ls4540\Documents\dev\households-over-the-years\output\five-decade-tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0225809E-1581-4B95-89D1-FF3D95DEAD10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF38E17E-9936-402C-AFFE-15289DB066ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -682,22 +682,22 @@
         <v>16</v>
       </c>
       <c r="B12" s="2">
-        <v>1.4489706619672309</v>
+        <v>1.661357834887111</v>
       </c>
       <c r="C12" s="2">
-        <v>1.3001323200205761</v>
+        <v>1.422404169346311</v>
       </c>
       <c r="D12" s="2">
-        <v>1.3113382692928499</v>
+        <v>1.444920606147754</v>
       </c>
       <c r="E12" s="2">
-        <v>1.3571921642244751</v>
+        <v>1.4837343922079429</v>
       </c>
       <c r="F12" s="2">
-        <v>1.1649366706834281</v>
+        <v>1.265752816410149</v>
       </c>
       <c r="G12" s="2">
-        <v>1.1450746275413071</v>
+        <v>1.192847439194354</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -705,22 +705,22 @@
         <v>17</v>
       </c>
       <c r="B13" s="2">
-        <v>1.3731170510574131</v>
+        <v>1.630645271810919</v>
       </c>
       <c r="C13" s="2">
-        <v>1.1685443888168421</v>
+        <v>1.409434849150369</v>
       </c>
       <c r="D13" s="2">
-        <v>1.092051603444085</v>
+        <v>1.388042680153873</v>
       </c>
       <c r="E13" s="2">
-        <v>1.0702563044192721</v>
+        <v>1.4417652820389359</v>
       </c>
       <c r="F13" s="2">
-        <v>0.96864856806077482</v>
+        <v>1.2241438726941041</v>
       </c>
       <c r="G13" s="2">
-        <v>0.98664927798589885</v>
+        <v>1.215529022564628</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -728,22 +728,22 @@
         <v>18</v>
       </c>
       <c r="B14" s="2">
-        <v>1.2566659547877801</v>
+        <v>1.515230375470672</v>
       </c>
       <c r="C14" s="2">
-        <v>1.078830418199842</v>
+        <v>1.330673039700353</v>
       </c>
       <c r="D14" s="2">
-        <v>0.97835946412118557</v>
+        <v>1.303503596270055</v>
       </c>
       <c r="E14" s="2">
-        <v>0.98991300655110237</v>
+        <v>1.339613118627704</v>
       </c>
       <c r="F14" s="2">
-        <v>0.91450836055197615</v>
+        <v>1.1735521566204909</v>
       </c>
       <c r="G14" s="2">
-        <v>0.93843066158578925</v>
+        <v>1.193804556958014</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -751,22 +751,22 @@
         <v>19</v>
       </c>
       <c r="B15" s="2">
-        <v>1.140409289761884</v>
+        <v>1.4122579958632311</v>
       </c>
       <c r="C15" s="2">
-        <v>0.99371944610348117</v>
+        <v>1.2614616907777969</v>
       </c>
       <c r="D15" s="2">
-        <v>0.91364556294567356</v>
+        <v>1.194721283851641</v>
       </c>
       <c r="E15" s="2">
-        <v>0.90805026798991917</v>
+        <v>1.210480221581268</v>
       </c>
       <c r="F15" s="2">
-        <v>0.85398956557666439</v>
+        <v>1.088221520620491</v>
       </c>
       <c r="G15" s="2">
-        <v>0.87927115589464355</v>
+        <v>1.136341803393238</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>